<commit_message>
Revert "Modified to work better for wind and nav."
This reverts commit d9d73383e7eb0e71b20c81427d467c5c3aca7829.
</commit_message>
<xml_diff>
--- a/Calls.xlsx
+++ b/Calls.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10517"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11207"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/fgorina/PlatformIO/Projects/Autopilot2000/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/fgorina/Desenvolopament_X/PlatformIO/Projects/Autopilot2000/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0623A3D7-3C1F-4845-A370-1375A1B87A2C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{4AB36928-D53C-2342-8DAD-9ECFAE020890}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="6920" yWindow="2100" windowWidth="28040" windowHeight="17440" xr2:uid="{3FA691A1-C58B-264E-AB79-CE9D70E677EA}"/>
+    <workbookView xWindow="37280" yWindow="12740" windowWidth="28040" windowHeight="17440" xr2:uid="{3FA691A1-C58B-264E-AB79-CE9D70E677EA}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -736,8 +736,7 @@
   <cols>
     <col min="1" max="1" width="24.83203125" customWidth="1"/>
     <col min="2" max="2" width="26.33203125" customWidth="1"/>
-    <col min="3" max="3" width="47.83203125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="28.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.83203125" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="45.1640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>

</xml_diff>